<commit_message>
Drop unverified MMUCC element numbers; note partial MMUCC 6th ed. upload
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RUF2qbndEzSEPvZD9nL4yj
</commit_message>
<xml_diff>
--- a/SCDOT_AASHTOWare_Safety_Treatments_and_Countermeasures_v8.xlsx
+++ b/SCDOT_AASHTOWare_Safety_Treatments_and_Countermeasures_v8.xlsx
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4004" uniqueCount="957">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4004" uniqueCount="956">
   <si>
     <t xml:space="preserve">Treatments &amp; Countermeasures</t>
   </si>
@@ -2666,7 +2666,7 @@
     <t xml:space="preserve">Values used in this workbook (SMS code)</t>
   </si>
   <si>
-    <t xml:space="preserve">New TR-310 / MMUCC 5th equivalent</t>
+    <t xml:space="preserve">New TR-310 / MMUCC equivalent</t>
   </si>
   <si>
     <t xml:space="preserve">Source / status</t>
@@ -2693,7 +2693,7 @@
     <t xml:space="preserve">Non Collision (00), Rear End (10), Head On (20), Angle (41/42/43), Sideswipe, Same Direction (50), Sideswipe, Opposite Direction (60)</t>
   </si>
   <si>
-    <t xml:space="preserve">C9 Manner of Crash: Front to Rear, Front to Front, Angle, Sideswipe... New-form codes differ (Angle is 80 there, not in the SMS)</t>
+    <t xml:space="preserve">Manner of Crash/Collision: Front to Rear, Front to Front, Angle, Sideswipe... New-form codes differ (Angle is 80 there, not in the SMS)</t>
   </si>
   <si>
     <t xml:space="preserve">Confirmed: your query + SC dictionary. Angle may list three times.</t>
@@ -2705,7 +2705,7 @@
     <t xml:space="preserve">Cross Median/Center (02), Overturn/Rollover (08), Ran off Road Left (09), Ran off Road Right (10), Animal - Deer (20), Animal - Other (21), Pedalcycle (26), Pedestrian (27), Bridge Parapet End (41), Bridge Pier or Abutment (42), Bridge Rail (43), Culvert (44), Ditch (46), Embankment (47), Guardrail End (50), Guardrail Face (51), Median Barrier (56), Tree (60), Utility Pole (61)</t>
   </si>
   <si>
-    <t xml:space="preserve">C7 First Harmful Event. Under MMUCC, ran off road and cross median are NOT harmful events - they only go in Sequence of Events. New-form codes differ (Pedestrian 26, Pedalcycle 25).</t>
+    <t xml:space="preserve">First Harmful Event. Under MMUCC, ran off road and cross median are NOT harmful events - they only go in Sequence of Events. New-form codes differ (Pedestrian 26, Pedalcycle 25).</t>
   </si>
   <si>
     <t xml:space="preserve">Confirmed: SC dictionary. Crash Harmful Event = most harmful event of the crash.</t>
@@ -2720,9 +2720,6 @@
     <t xml:space="preserve">Same list as above. Used here: Cross Median/Center, Ran off Road Left</t>
   </si>
   <si>
-    <t xml:space="preserve">V20 Sequence of Events</t>
-  </si>
-  <si>
     <t xml:space="preserve">Use with '=' only. '≠' drops that row, not the crash.</t>
   </si>
   <si>
@@ -2732,7 +2729,7 @@
     <t xml:space="preserve">Gore (1), Island (2), Median (3), Roadside (4), Roadway (5), Shoulder (6), Sidewalk (7), Outside Trafficway (8), Unknown (9)</t>
   </si>
   <si>
-    <t xml:space="preserve">C8 Location of First Harmful Event</t>
+    <t xml:space="preserve">Location of First Harmful Event Relative to the Trafficway</t>
   </si>
   <si>
     <t xml:space="preserve">Confirmed: SMS dictionary you sent</t>
@@ -36363,95 +36360,95 @@
         <v>846</v>
       </c>
       <c r="D6" s="29" t="s">
+        <v>844</v>
+      </c>
+      <c r="E6" s="29" t="s">
         <v>847</v>
-      </c>
-      <c r="E6" s="29" t="s">
-        <v>848</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="30" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="B7" s="29" t="s">
         <v>832</v>
       </c>
       <c r="C7" s="29" t="s">
+        <v>849</v>
+      </c>
+      <c r="D7" s="29" t="s">
         <v>850</v>
       </c>
-      <c r="D7" s="29" t="s">
+      <c r="E7" s="29" t="s">
         <v>851</v>
-      </c>
-      <c r="E7" s="29" t="s">
-        <v>852</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="30" t="s">
+        <v>852</v>
+      </c>
+      <c r="B8" s="29" t="s">
         <v>853</v>
       </c>
-      <c r="B8" s="29" t="s">
+      <c r="C8" s="29" t="s">
         <v>854</v>
       </c>
-      <c r="C8" s="29" t="s">
+      <c r="D8" s="29" t="s">
         <v>855</v>
       </c>
-      <c r="D8" s="29" t="s">
+      <c r="E8" s="29" t="s">
         <v>856</v>
-      </c>
-      <c r="E8" s="29" t="s">
-        <v>857</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="30" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="B9" s="29" t="s">
         <v>832</v>
       </c>
       <c r="C9" s="29" t="s">
+        <v>858</v>
+      </c>
+      <c r="D9" s="29" t="s">
         <v>859</v>
       </c>
-      <c r="D9" s="29" t="s">
+      <c r="E9" s="29" t="s">
         <v>860</v>
-      </c>
-      <c r="E9" s="29" t="s">
-        <v>861</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="30" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="B10" s="29" t="s">
         <v>832</v>
       </c>
       <c r="C10" s="29" t="s">
+        <v>862</v>
+      </c>
+      <c r="D10" s="29" t="s">
         <v>863</v>
       </c>
-      <c r="D10" s="29" t="s">
-        <v>864</v>
-      </c>
       <c r="E10" s="29" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="30" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="B11" s="29" t="s">
         <v>832</v>
       </c>
       <c r="C11" s="29" t="s">
+        <v>865</v>
+      </c>
+      <c r="D11" s="29" t="s">
         <v>866</v>
       </c>
-      <c r="D11" s="29" t="s">
+      <c r="E11" s="29" t="s">
         <v>867</v>
-      </c>
-      <c r="E11" s="29" t="s">
-        <v>868</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -36462,159 +36459,159 @@
         <v>832</v>
       </c>
       <c r="C12" s="29" t="s">
+        <v>868</v>
+      </c>
+      <c r="D12" s="29" t="s">
         <v>869</v>
       </c>
-      <c r="D12" s="29" t="s">
+      <c r="E12" s="29" t="s">
         <v>870</v>
-      </c>
-      <c r="E12" s="29" t="s">
-        <v>871</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="30" t="s">
+        <v>871</v>
+      </c>
+      <c r="B13" s="29" t="s">
         <v>872</v>
       </c>
-      <c r="B13" s="29" t="s">
+      <c r="C13" s="29" t="s">
         <v>873</v>
       </c>
-      <c r="C13" s="29" t="s">
+      <c r="D13" s="29" t="s">
         <v>874</v>
       </c>
-      <c r="D13" s="29" t="s">
+      <c r="E13" s="29" t="s">
         <v>875</v>
-      </c>
-      <c r="E13" s="29" t="s">
-        <v>876</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="30" t="s">
+        <v>876</v>
+      </c>
+      <c r="B14" s="29" t="s">
+        <v>872</v>
+      </c>
+      <c r="C14" s="29" t="s">
         <v>877</v>
       </c>
-      <c r="B14" s="29" t="s">
-        <v>873</v>
-      </c>
-      <c r="C14" s="29" t="s">
+      <c r="D14" s="29" t="s">
         <v>878</v>
       </c>
-      <c r="D14" s="29" t="s">
+      <c r="E14" s="29" t="s">
         <v>879</v>
-      </c>
-      <c r="E14" s="29" t="s">
-        <v>880</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="30" t="s">
+        <v>880</v>
+      </c>
+      <c r="B15" s="29" t="s">
+        <v>872</v>
+      </c>
+      <c r="C15" s="29" t="s">
         <v>881</v>
       </c>
-      <c r="B15" s="29" t="s">
-        <v>873</v>
-      </c>
-      <c r="C15" s="29" t="s">
+      <c r="D15" s="29" t="s">
         <v>882</v>
       </c>
-      <c r="D15" s="29" t="s">
+      <c r="E15" s="29" t="s">
         <v>883</v>
-      </c>
-      <c r="E15" s="29" t="s">
-        <v>884</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="30" t="s">
+        <v>884</v>
+      </c>
+      <c r="B16" s="29" t="s">
         <v>885</v>
       </c>
-      <c r="B16" s="29" t="s">
+      <c r="C16" s="29" t="s">
         <v>886</v>
       </c>
-      <c r="C16" s="29" t="s">
+      <c r="D16" s="29" t="s">
         <v>887</v>
       </c>
-      <c r="D16" s="29" t="s">
+      <c r="E16" s="29" t="s">
         <v>888</v>
-      </c>
-      <c r="E16" s="29" t="s">
-        <v>889</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="30" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="B17" s="29" t="s">
         <v>832</v>
       </c>
       <c r="C17" s="29" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="D17" s="29" t="s">
         <v>126</v>
       </c>
       <c r="E17" s="29" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="30" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="B18" s="29" t="s">
         <v>832</v>
       </c>
       <c r="C18" s="29" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="D18" s="29" t="s">
         <v>126</v>
       </c>
       <c r="E18" s="29" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="30" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="B19" s="29" t="s">
         <v>832</v>
       </c>
       <c r="C19" s="29" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="D19" s="29" t="s">
         <v>126</v>
       </c>
       <c r="E19" s="29" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="30" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="B20" s="29" t="s">
         <v>832</v>
       </c>
       <c r="C20" s="29" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="D20" s="29" t="s">
         <v>126</v>
       </c>
       <c r="E20" s="29" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="61" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="B23" s="61"/>
       <c r="C23" s="61"/>
@@ -36623,7 +36620,7 @@
     </row>
     <row r="24" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="61" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="B24" s="61"/>
       <c r="C24" s="61"/>
@@ -36632,7 +36629,7 @@
     </row>
     <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="61" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="B25" s="61"/>
       <c r="C25" s="61"/>
@@ -36641,7 +36638,7 @@
     </row>
     <row r="26" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="61" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="B26" s="61"/>
       <c r="C26" s="61"/>
@@ -36650,7 +36647,7 @@
     </row>
     <row r="27" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="61" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -36691,7 +36688,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -36699,76 +36696,76 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="62" t="s">
+        <v>907</v>
+      </c>
+      <c r="B2" s="62" t="s">
         <v>908</v>
       </c>
-      <c r="B2" s="62" t="s">
+      <c r="C2" s="62" t="s">
         <v>909</v>
       </c>
-      <c r="C2" s="62" t="s">
+      <c r="D2" s="62" t="s">
         <v>910</v>
-      </c>
-      <c r="D2" s="62" t="s">
-        <v>911</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="30" t="s">
+        <v>911</v>
+      </c>
+      <c r="B3" s="29" t="s">
         <v>912</v>
       </c>
-      <c r="B3" s="29" t="s">
+      <c r="C3" s="29" t="s">
         <v>913</v>
-      </c>
-      <c r="C3" s="29" t="s">
-        <v>914</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="78.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="30" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="B4" s="29" t="s">
+        <v>914</v>
+      </c>
+      <c r="C4" s="29" t="s">
         <v>915</v>
-      </c>
-      <c r="C4" s="29" t="s">
-        <v>916</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="30" t="s">
+        <v>916</v>
+      </c>
+      <c r="B5" s="29" t="s">
         <v>917</v>
       </c>
-      <c r="B5" s="29" t="s">
+      <c r="C5" s="29" t="s">
         <v>918</v>
-      </c>
-      <c r="C5" s="29" t="s">
-        <v>919</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="30" t="s">
+        <v>919</v>
+      </c>
+      <c r="B6" s="29" t="s">
         <v>920</v>
       </c>
-      <c r="B6" s="29" t="s">
+      <c r="C6" s="29" t="s">
         <v>921</v>
-      </c>
-      <c r="C6" s="29" t="s">
-        <v>922</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="30" t="s">
+        <v>922</v>
+      </c>
+      <c r="B7" s="29" t="s">
         <v>923</v>
       </c>
-      <c r="B7" s="29" t="s">
+      <c r="C7" s="29" t="s">
         <v>924</v>
-      </c>
-      <c r="C7" s="29" t="s">
-        <v>925</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -36782,7 +36779,7 @@
         <v>129</v>
       </c>
       <c r="D10" s="63" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -36794,7 +36791,7 @@
       </c>
       <c r="C11" s="29"/>
       <c r="D11" s="63" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -36806,7 +36803,7 @@
       </c>
       <c r="C12" s="29"/>
       <c r="D12" s="63" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -36820,7 +36817,7 @@
         <v>144</v>
       </c>
       <c r="D13" s="63" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -36832,7 +36829,7 @@
       </c>
       <c r="C14" s="29"/>
       <c r="D14" s="63" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -36846,7 +36843,7 @@
         <v>155</v>
       </c>
       <c r="D15" s="63" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -36860,7 +36857,7 @@
         <v>160</v>
       </c>
       <c r="D16" s="63" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="91.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -36874,7 +36871,7 @@
         <v>167</v>
       </c>
       <c r="D17" s="63" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -36888,7 +36885,7 @@
         <v>171</v>
       </c>
       <c r="D18" s="63" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="129" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -36902,7 +36899,7 @@
         <v>179</v>
       </c>
       <c r="D19" s="63" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="91.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -36914,7 +36911,7 @@
       </c>
       <c r="C20" s="29"/>
       <c r="D20" s="63" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="129" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -36926,7 +36923,7 @@
       </c>
       <c r="C21" s="29"/>
       <c r="D21" s="63" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="116.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -36940,7 +36937,7 @@
         <v>194</v>
       </c>
       <c r="D22" s="63" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="178.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -36954,7 +36951,7 @@
         <v>199</v>
       </c>
       <c r="D23" s="63" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="141" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -36968,7 +36965,7 @@
         <v>204</v>
       </c>
       <c r="D24" s="63" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -36980,7 +36977,7 @@
       </c>
       <c r="C25" s="29"/>
       <c r="D25" s="63" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -36992,7 +36989,7 @@
       </c>
       <c r="C26" s="29"/>
       <c r="D26" s="63" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -37000,11 +36997,11 @@
         <v>210</v>
       </c>
       <c r="B27" s="29" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="C27" s="29"/>
       <c r="D27" s="63" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -37018,7 +37015,7 @@
         <v>218</v>
       </c>
       <c r="D28" s="63" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="78.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -37032,7 +37029,7 @@
         <v>223</v>
       </c>
       <c r="D29" s="63" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="91.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -37040,11 +37037,11 @@
         <v>224</v>
       </c>
       <c r="B30" s="29" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="C30" s="29"/>
       <c r="D30" s="63" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -37052,11 +37049,11 @@
         <v>226</v>
       </c>
       <c r="B31" s="29" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="C31" s="29"/>
       <c r="D31" s="63" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -37070,7 +37067,7 @@
         <v>233</v>
       </c>
       <c r="D32" s="63" t="s">
-        <v>949</v>
+        <v>948</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -37082,7 +37079,7 @@
       </c>
       <c r="C33" s="29"/>
       <c r="D33" s="63" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -37090,13 +37087,13 @@
         <v>237</v>
       </c>
       <c r="B34" s="29" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="C34" s="29" t="s">
         <v>241</v>
       </c>
       <c r="D34" s="63" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -37104,11 +37101,11 @@
         <v>242</v>
       </c>
       <c r="B35" s="29" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="C35" s="29"/>
       <c r="D35" s="63" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -37122,7 +37119,7 @@
         <v>248</v>
       </c>
       <c r="D36" s="63" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -37136,7 +37133,7 @@
         <v>253</v>
       </c>
       <c r="D37" s="63" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -37150,7 +37147,7 @@
         <v>259</v>
       </c>
       <c r="D38" s="63" t="s">
-        <v>955</v>
+        <v>954</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="129" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -37162,7 +37159,7 @@
       </c>
       <c r="C39" s="29"/>
       <c r="D39" s="63" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add MMUCC 6th edition version of the 30 criteria; verify field mappings
- New sheet: same criteria on MMUCC 6 fields plus rebuilt derived fields
- Field Reference MMUCC column now cites verified 6th ed. elements
- Median Barriers: flag interchange-area coding (Non-Junction gap)
- Notes: section 9 on what MMUCC 6 confirms and changes

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RUF2qbndEzSEPvZD9nL4yj
</commit_message>
<xml_diff>
--- a/SCDOT_AASHTOWare_Safety_Treatments_and_Countermeasures_v8.xlsx
+++ b/SCDOT_AASHTOWare_Safety_Treatments_and_Countermeasures_v8.xlsx
@@ -13,7 +13,8 @@
     <sheet name="Countermeasures" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Treatments" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Field Reference" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Changes" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="New TR-310 (MMUCC 6)" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Changes" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Countermeasures!$A$3:$K$33</definedName>
@@ -66,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4004" uniqueCount="956">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4115" uniqueCount="1032">
   <si>
     <t xml:space="preserve">Treatments &amp; Countermeasures</t>
   </si>
@@ -698,7 +699,7 @@
     <t xml:space="preserve">Trafficway drops undivided roads (centerline crashes), one-way ramps and roads that already have a barrier (I-20 crash 23239996). First Harmful Event Location = Median brings in every object in the median - piers, abutments, walls, poles, ditches - in one line. 'First Harmful Event ≠ Ran off Road Right' replaced with Location ≠ Roadside so a driver who goes right, overcorrects and crosses the median stays in. AADT &gt; 20,000 matches AASHTO RDG Fig. 6-1.</t>
   </si>
   <si>
-    <t xml:space="preserve">Median width (30 ft or less per RDG) is not in the crash data - check against inventory. Wrong-way head-ons can't be removed with crash-level fields. CMF 7040 (0.03) is cross-median only.</t>
+    <t xml:space="preserve">Check whether Junction Type has interchange or ramp values: freeway crashes inside an interchange may not be NON-JUNCTION. Median width (30 ft or less per RDG) is not in the crash data - check against inventory. Wrong-way head-ons can't be removed with crash-level fields. CMF 7040 (0.03) is cross-median only.</t>
   </si>
   <si>
     <t xml:space="preserve">CM: Roadside Design Improvements at Curves</t>
@@ -2666,7 +2667,7 @@
     <t xml:space="preserve">Values used in this workbook (SMS code)</t>
   </si>
   <si>
-    <t xml:space="preserve">New TR-310 / MMUCC equivalent</t>
+    <t xml:space="preserve">New TR-310: MMUCC 6th ed. element (DOT HS 813 525, Feb 2025)</t>
   </si>
   <si>
     <t xml:space="preserve">Source / status</t>
@@ -2681,7 +2682,7 @@
     <t xml:space="preserve">NON-JUNCTION (13), Cross-Over (01), Driveway (02), Four-Way Intersection (04), T-Intersection (08), Y-Intersection (12), Five/More Points (03), Traffic Circle (09)</t>
   </si>
   <si>
-    <t xml:space="preserve">Split into Relation to Junction + Type of Intersection</t>
+    <t xml:space="preserve">C12 Relation to Junction (Specific Location: Non-Junction, Intersection or Related, Driveway Access or Related, Crossover-Related, Entrance or Exit Ramp or Related, Through Roadway, Other Location Within an Interchange Area...) + C13 Type of Intersection (T, Y, L, Four-Leg, Five or More Legs, Circular, Other e.g. RCUT)</t>
   </si>
   <si>
     <t xml:space="preserve">Confirmed: your Condition Builder query + SC crash data dictionary</t>
@@ -2693,7 +2694,7 @@
     <t xml:space="preserve">Non Collision (00), Rear End (10), Head On (20), Angle (41/42/43), Sideswipe, Same Direction (50), Sideswipe, Opposite Direction (60)</t>
   </si>
   <si>
-    <t xml:space="preserve">Manner of Crash/Collision: Front to Rear, Front to Front, Angle, Sideswipe... New-form codes differ (Angle is 80 there, not in the SMS)</t>
+    <t xml:space="preserve">C9 Manner of Collision of the First Harmful Event: Not a Collision With a MV In-Transport, Angle, Front to Front, Front-to-Rear or Rear-to-Front, Rear to Rear, Rear-to-Side, Sideswipe Opposite / Same Direction</t>
   </si>
   <si>
     <t xml:space="preserve">Confirmed: your query + SC dictionary. Angle may list three times.</t>
@@ -2705,7 +2706,7 @@
     <t xml:space="preserve">Cross Median/Center (02), Overturn/Rollover (08), Ran off Road Left (09), Ran off Road Right (10), Animal - Deer (20), Animal - Other (21), Pedalcycle (26), Pedestrian (27), Bridge Parapet End (41), Bridge Pier or Abutment (42), Bridge Rail (43), Culvert (44), Ditch (46), Embankment (47), Guardrail End (50), Guardrail Face (51), Median Barrier (56), Tree (60), Utility Pole (61)</t>
   </si>
   <si>
-    <t xml:space="preserve">First Harmful Event. Under MMUCC, ran off road and cross median are NOT harmful events - they only go in Sequence of Events. New-form codes differ (Pedestrian 26, Pedalcycle 25).</t>
+    <t xml:space="preserve">C7 First Harmful Event. No ran-off-road or cross-median values. Non-Motorist covers peds and bikes; Live Animal has no deer split. No crash-level 'most harmful event' - V38 is per vehicle.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirmed: SC dictionary. Crash Harmful Event = most harmful event of the crash.</t>
@@ -2720,6 +2721,9 @@
     <t xml:space="preserve">Same list as above. Used here: Cross Median/Center, Ran off Road Left</t>
   </si>
   <si>
+    <t xml:space="preserve">V37 Sequence of Events (per vehicle, multi-select): Cross Centerline, Cross Median, Ran Off Roadway Left / Right / Direction Unknown, Re-Entering Roadway...</t>
+  </si>
+  <si>
     <t xml:space="preserve">Use with '=' only. '≠' drops that row, not the crash.</t>
   </si>
   <si>
@@ -2729,7 +2733,7 @@
     <t xml:space="preserve">Gore (1), Island (2), Median (3), Roadside (4), Roadway (5), Shoulder (6), Sidewalk (7), Outside Trafficway (8), Unknown (9)</t>
   </si>
   <si>
-    <t xml:space="preserve">Location of First Harmful Event Relative to the Trafficway</t>
+    <t xml:space="preserve">C8 Location of First Harmful Event: On Roadway, Continuous Left-Turn Lane, On Shoulder, On Roadside, On Median, Pedestrian Refuge Island or Traffic Island, In Parking Lane, Separator, Gore, Non-Trafficway Area</t>
   </si>
   <si>
     <t xml:space="preserve">Confirmed: SMS dictionary you sent</t>
@@ -2744,7 +2748,7 @@
     <t xml:space="preserve">Two-Way, Not Divided (1); Two-Way, Divided, Unprotected Median (2); Two-Way, Divided, Barrier (3); One-Way (4); Other (8)</t>
   </si>
   <si>
-    <t xml:space="preserve">Trafficway Description (adds TWLTL as its own value)</t>
+    <t xml:space="preserve">V25 Trafficway Flow (One-Way, Two-Way, Two-Way With a Continuous Left-Turn Lane) + V26 Median Barrier Presence (Not Applicable - no median; Median Without a Traffic Barrier; Median With Traffic Barrier). Both per vehicle.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirmed: SMS dictionary + SC dictionary. Under Roadway, next to AADT.</t>
@@ -2756,7 +2760,7 @@
     <t xml:space="preserve">Curve-Level (4), Curve-On Grade (5), Curve-Hillcrest (6)</t>
   </si>
   <si>
-    <t xml:space="preserve">Roadway Alignment and Grade (Curve Left / Curve Right)</t>
+    <t xml:space="preserve">V28 Roadway Alignment (Straight, Curve Left, Curve Right) + V29 Roadway Grade. Per vehicle.</t>
   </si>
   <si>
     <t xml:space="preserve">SC dictionary - confirm dropdown label</t>
@@ -2768,7 +2772,7 @@
     <t xml:space="preserve">Dark (Lighting Unspecified) (4), Dark (Street Lamp Lit) (5), Dark (Street Lamps Not Lit) (6), Dark (No Lights) (7)</t>
   </si>
   <si>
-    <t xml:space="preserve">Light Condition: Dark-Lighted, Dark-Not Lighted, Dark-Unknown Lighting</t>
+    <t xml:space="preserve">C11 Light Condition: Dark - Lighted, Dark - Not Lighted, Dark - Unknown Lighting</t>
   </si>
   <si>
     <t xml:space="preserve">Road Surface Condition</t>
@@ -2777,7 +2781,7 @@
     <t xml:space="preserve">Wet (2)</t>
   </si>
   <si>
-    <t xml:space="preserve">Roadway Surface Condition</t>
+    <t xml:space="preserve">V30 Roadway Surface Condition (per vehicle): Wet. Water (standing or moving) is separate.</t>
   </si>
   <si>
     <t xml:space="preserve">SC dictionary</t>
@@ -2786,7 +2790,7 @@
     <t xml:space="preserve">Traffic Signal, Stop Sign</t>
   </si>
   <si>
-    <t xml:space="preserve">Traffic Control Device Type</t>
+    <t xml:space="preserve">V31 Traffic Control Device (per vehicle): Stop Sign, Traffic Control Signal, Flashing Traffic Control Signal...</t>
   </si>
   <si>
     <t xml:space="preserve">Label not confirmed - check dropdown</t>
@@ -2801,7 +2805,7 @@
     <t xml:space="preserve">Disregarded Sign/Signal (01), Exceeded Speed Limit (04), Obstruction in Roadway, Debris. Too Fast for Conditions (03) not used.</t>
   </si>
   <si>
-    <t xml:space="preserve">Driver Contributing Circumstances + Speeding-Related (Racing / Exceeded / Too Fast)</t>
+    <t xml:space="preserve">Split in three: D5 Speeding-Related (Yes, Racing / Exceeded Speed Limit / Too Fast for Conditions); D10 Related Factors - Driver Level (Failure to Obey Traffic Control Devices, Overcorrecting...); C17 Related Factors - Crash Level (Obstruction in Roadway). No 'Debris' value.</t>
   </si>
   <si>
     <t xml:space="preserve">Codes 01/03/04 from SC dictionary; roadway labels from the team meeting. '≠' works on run-off-road crashes because they have one unit.</t>
@@ -2813,7 +2817,7 @@
     <t xml:space="preserve">Pedalcycle, Pedestrian</t>
   </si>
   <si>
-    <t xml:space="preserve">Unit Type / Non-Motorist Unit Type</t>
+    <t xml:space="preserve">P5 Person Type (Pedestrian..., Bicyclist, Other Cyclist) + NM9 Non-Motorist Device Type</t>
   </si>
   <si>
     <t xml:space="preserve">Numetric filter logic</t>
@@ -2825,7 +2829,7 @@
     <t xml:space="preserve">Turning Left</t>
   </si>
   <si>
-    <t xml:space="preserve">Vehicle Maneuver/Action</t>
+    <t xml:space="preserve">V33 Vehicle Status Prior to Critical Event: Turning Left, Turning Right, Negotiating a Curve...</t>
   </si>
   <si>
     <t xml:space="preserve">Field name not confirmed - check builder</t>
@@ -2840,7 +2844,7 @@
     <t xml:space="preserve">AADT &gt; 20000 / &lt;= 20000, Through Lanes = 2 / = 4 / &gt;= 4, Speed Limit &gt;= 35 / &lt;= 40, Area Type = Urban / Rural</t>
   </si>
   <si>
-    <t xml:space="preserve">Not crash-report fields (road inventory)</t>
+    <t xml:space="preserve">AADT and area type are not on the report (link to road inventory, Ch. 10). Speed limit is V24 and lanes are V27 Number of Open Lanes, both per vehicle.</t>
   </si>
   <si>
     <t xml:space="preserve">AADT and lanes confirmed under Roadway. Speed Limit and Area Type - confirm.</t>
@@ -2894,7 +2898,338 @@
     <t xml:space="preserve">4. Pick values from the dropdown. Codes here are only to check the JSON / export. The SMS codes are not the new TR-310 codes (Pedestrian is 27 in the SMS, 26 on the new form).</t>
   </si>
   <si>
-    <t xml:space="preserve">5. New-form (MMUCC) crash reports are not in production yet. When they load, ran off road and cross median will be in Sequence of Events only, so criteria that look for them in First Harmful Event will start missing crashes.</t>
+    <t xml:space="preserve">5. New-form (MMUCC) crash reports are not in production yet. When they load: ran off road, cross median and cross centerline exist only in Sequence of Events; First Harmful Event has one 'Non-Motorist' value for pedestrians and bicyclists; and Non-Junction leaves out crashes inside interchange areas. See the 'New TR-310 (MMUCC 6)' sheet.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6. In MMUCC 6 the road conditions (surface, alignment, traffic control, speed limit, lanes, trafficway flow, median barrier) are recorded per vehicle, so rule 3 applies to them too.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SAME CRITERIA ON THE NEW TR-310 (MMUCC 6TH EDITION FIELDS)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">For when new-form reports reach production. Field names are MMUCC's (DOT HS 813 525, Feb 2025); SC's dropdown labels may differ. 'Pedestrian', 'Bicyclist' and 'Segment' are defined in the first block.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Derived field</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rebuilt on MMUCC 6 fields</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Note</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manner of Collision = The First Harmful Event Was Not a Collision With a Motor Vehicle In-Transport
+AND First Harmful Event ≠ Non-Motorist
+AND First Harmful Event ≠ Live Animal
+AND First Harmful Event ≠ Ridden Animal or Animal-Drawn Conveyance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deer and other animals are one attribute (Live Animal) in MMUCC 6.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Roadway Departure = Yes
+OR Manner of Collision = Front to Front
+OR Manner of Collision = Sideswipe, Opposite Direction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'Head On' is called Front to Front.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Intersection Related</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relation to Junction = Intersection or Related</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Type of Intersection (C13) gives the shape. Driveways are their own value (Driveway Access or Related).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First Harmful Event = Non-Motorist
+AND (   Person Type = Pedestrian Walking, Running, Jogging, Hiking, Sitting, Lying
+     OR Person Type = Pedestrian on Personal Conveyance )</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First Harmful Event no longer splits pedestrian and bicycle - Person Type (P5) does.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bicyclist</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Person Type = Bicyclist OR Person Type = Other Cyclist</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Or Non-Motorist Device Type (NM9) = Bicycle / Other Cycle.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Segment (non-intersection)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relation to Junction = Non-Junction, Through Roadway
+                       or Other Location Within an Interchange Area</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In MMUCC 6, Non-Junction only covers crashes OUTSIDE an interchange area. Freeway mainline crashes inside an interchange are Through Roadway; median/shoulder/roadside ones are Other Location Within an Interchange Area.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crash criteria on MMUCC 6 fields</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What changes / new options</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Speeding-Related = Yes, Exceeded Speed Limit
+ OR Speeding-Related = Yes, Racing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Too Fast for Conditions is its own attribute (D5), so the team's decision maps one to one.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bicyclist = Yes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New option: Non-Motorist Specific Location (NM7) = In Painted Cycle Lane / In Physically Separated Cycle Lane shows whether a bike lane was already there.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pedestrian = Yes
+AND Intersection Related = Yes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New option: Non-Motorist in Crosswalk (NM6) = Yes, Marked / Yes, Unmarked, and Non-Motorist Status (NM2) = Crossing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pedestrian = Yes
+AND Intersection Related = Yes
+AND Traffic Control Device = Traffic Control Signal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Traffic Control Device (V31) is per vehicle; '=' works. New option: Non-Motorist Traffic Control Device (NM10) = Non-Motorist Crossing Signal - an LPI needs pedestrian signal heads.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pedestrian = Yes
+AND Relation to Junction ≠ Intersection or Related
+AND Area Type = Urban
+AND Through Lanes &gt;= 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lanes still from road inventory (V27 counts one direction only on divided roads). New option: NM2 = Crossing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pedestrian = Yes
+AND Relation to Junction ≠ Intersection or Related
+AND Traffic Control Device ≠ Traffic Control Signal
+AND (   Motor Vehicle Posted or Statutory Speed Limit &gt;= 35
+     OR Through Lanes &gt;= 4 )</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Speed limit is now on the crash report (V24, per vehicle). New option: NM2 = Crossing, NM10 = None.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pedestrian = Yes
+AND Relation to Junction ≠ Intersection or Related
+AND Traffic Control Device ≠ Traffic Control Signal
+AND Motor Vehicle Posted or Statutory Speed Limit &lt;= 40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same options as PHB.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Area Type = Urban
+AND Median Barrier Presence = Not Applicable (no median)
+AND Trafficway Flow = Two-Way
+AND Number of Open Lanes = 4
+AND AADT &lt;= 20000
+AND (   Manner of Collision = Front-to-Rear or Rear-to-Front
+     OR Manner of Collision = Front to Front
+     OR Manner of Collision = Angle
+     OR Pedestrian = Yes
+     OR Bicyclist = Yes )</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trafficway Flow = Two-Way (not 'With a Continuous Left-Turn Lane') leaves out roads that are already three-lane. On an undivided road V27 counts both directions, so 4 = four-lane undivided.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pedestrian = Yes
+AND Relation to Junction ≠ Intersection or Related</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New option: NM2 = Movement Against Traffic / Movement With Traffic - the 'walking along the road' filter becomes possible.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lane Departure = Yes
+AND Relation to Junction = Non-Junction, Through Roadway
+                       or Other Location Within an Interchange Area
+AND Roadway Alignment = Curve Left or Curve Right
+AND Related Factors - Crash Level ≠ Obstruction in Roadway
+AND First Harmful Event ≠ Other Object (not fixed)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Curve Left / Curve Right exist again (V28, per vehicle). There is no 'Debris' attribute: debris hits are First Harmful Event = Other Object (not fixed).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lane Departure = Yes
+AND Roadway Departure = No
+AND Relation to Junction = Non-Junction
+AND Median Barrier Presence = Not Applicable (no median)
+AND Number of Open Lanes = 2
+AND Area Type = Rural</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New option: Sequence of Events = Cross Centerline brings in single-vehicle centerline crossings.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Roadway Departure = Yes
+AND Relation to Junction = Non-Junction, Through Roadway
+                       or Other Location Within an Interchange Area
+AND Area Type = Rural
+AND Related Factors - Crash Level ≠ Obstruction in Roadway
+AND First Harmful Event ≠ Other Object (not fixed)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New option: Sequence of Events = Ran Off Roadway Right.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relation to Junction = Non-Junction, Through Roadway
+                       or Other Location Within an Interchange Area
+AND Median Barrier Presence = Median Without a Traffic Barrier
+AND AADT &gt; 20000
+AND (   Manner of Collision = Front to Front
+     OR Manner of Collision = Sideswipe, Opposite Direction
+     OR Sequence of Events = Cross Median
+     OR Sequence of Events = Ran Off Roadway Left
+     OR Location of First Harmful Event = On Median )
+AND Location of First Harmful Event ≠ On Roadside
+AND Location of First Harmful Event ≠ Non-Trafficway Area</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Median Barrier Presence (V26) replaces Trafficway 2/3. Cross Median and Ran Off Roadway Left only exist in Sequence of Events. Without Through Roadway / Other Location Within an Interchange Area every freeway crash inside an interchange drops out. Manner of Collision is only for the FIRST harmful event, so a car that hits a median object and then an opposing car is caught by Sequence of Events, not by Front to Front. Wrong-way drivers: D10 has 'Driving on Wrong Side of Two-Way Trafficway', but it is a driver field, so '≠' won't remove the crash.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Roadway Departure = Yes
+AND Relation to Junction = Non-Junction, Through Roadway
+                       or Other Location Within an Interchange Area
+AND Roadway Alignment = Curve Left or Curve Right
+AND (   Location of First Harmful Event = On Roadside
+     OR Location of First Harmful Event = On Shoulder )
+AND Related Factors - Crash Level ≠ Obstruction in Roadway
+AND First Harmful Event ≠ Other Object (not fixed)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Roadway Departure = Yes
+AND Relation to Junction = Non-Junction, Through Roadway
+                       or Other Location Within an Interchange Area
+AND (   Location of First Harmful Event = On Roadside
+     OR Location of First Harmful Event = On Shoulder )
+AND First Harmful Event ≠ Guardrail Face
+AND First Harmful Event ≠ Guardrail End
+AND First Harmful Event ≠ Concrete Traffic Barrier
+AND First Harmful Event ≠ Cable Barrier
+AND Related Factors - Crash Level ≠ Obstruction in Roadway
+AND First Harmful Event ≠ Other Object (not fixed)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MMUCC splits barriers into cable, concrete, guardrail face/end and other.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New option: Related Factors - Driver Level (D10) = Overcorrecting, which is the edge drop-off crash SafetyEdge targets.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Intersection Related = Yes
+AND Traffic Control Device = Traffic Control Signal
+AND (   Manner of Collision = Angle
+     OR Manner of Collision = Front-to-Rear or Rear-to-Front )</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(   Intersection Related = Yes
+ OR Relation to Junction = Driveway Access or Related )
+AND (   Manner of Collision = Angle
+     OR Manner of Collision = Front-to-Rear or Rear-to-Front
+     OR Manner of Collision = Front to Front )</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Intersection Related = Yes
+AND (   Manner of Collision = Front-to-Rear or Rear-to-Front
+     OR Manner of Collision = Angle )</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New option: Vehicle Status Prior to Critical Event (V33) = Turning Right.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Intersection Related = Yes
+AND (   Manner of Collision = Angle
+     OR Manner of Collision = Front-to-Rear or Rear-to-Front
+     OR Manner of Collision = Front to Front )</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New option: V33 = Turning Left.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Intersection Related = Yes
+AND (   Manner of Collision = Angle
+     OR Manner of Collision = Front to Front )</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New option: Median Barrier Presence = Median Without a Traffic Barrier (J-turns and RCUTs need a median). Existing RCUTs are Type of Intersection = Other Intersection Type.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Intersection Related = Yes
+AND Traffic Control Device = Traffic Control Signal
+AND (   Manner of Collision = Angle
+     OR Manner of Collision = Front to Front )
+AND Vehicle Status Prior to Critical Event = Turning Left</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Intersection Related = Yes
+AND Type of Intersection ≠ Circular Intersection
+AND (   Manner of Collision = Angle
+     OR Manner of Collision = Front to Front )</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Intersection Related = Yes
+AND Traffic Control Device = Stop Sign
+AND Manner of Collision = Angle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Intersection Related = Yes
+AND Traffic Control Device = Stop Sign
+AND Manner of Collision = Angle
+AND Area Type = Rural</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Traffic Control Device = Stop Sign
+AND (   Type of Intersection = T-Intersection
+     OR Type of Intersection = Y-Intersection
+     OR Type of Intersection = Four-Leg Intersection )</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MMUCC adds L-Intersection; left out here.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Intersection Related = Yes
+AND Traffic Control Device = Traffic Control Signal
+AND (   Manner of Collision = Front-to-Rear or Rear-to-Front
+     OR Manner of Collision = Angle )
+AND Related Factors - Driver Level = Failure to Obey Traffic Control Devices</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(   Light Condition = Dark - Not Lighted
+ OR Light Condition = Dark - Lighted
+ OR Light Condition = Dark - Unknown Lighting )
+AND Manner of Collision ≠ Front-to-Rear or Rear-to-Front</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MMUCC has three dark values; the SMS has four.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Roadway Surface Condition = Wet
+AND (   Roadway Departure = Yes
+     OR Roadway Alignment = Curve Left
+     OR Roadway Alignment = Curve Right )
+AND Related Factors - Crash Level ≠ Obstruction in Roadway
+AND First Harmful Event ≠ Other Object (not fixed)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Water (standing or moving) is its own attribute; left out - that is drainage, not friction.</t>
   </si>
   <si>
     <t xml:space="preserve">CHANGES FROM THE PREVIOUS VERSION</t>
@@ -2943,6 +3278,15 @@
   </si>
   <si>
     <t xml:space="preserve">AASHTOWare applies the CMF only to crashes that pass the countermeasure criteria. If the CMF was measured on a different group, the benefit is off. This is the 51% vs 13% problem from the meeting.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New sheet 'New TR-310 (MMUCC 6)'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The same 30 criteria written on MMUCC 6th edition fields.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SC's new TR-310 follows MMUCC. Checked against the MMUCC 6th edition (DOT HS 813 525, Feb 2025) so the criteria are ready when new-form reports reach production.</t>
   </si>
   <si>
     <t xml:space="preserve">Treatment Selector, column AA</t>
@@ -36262,7 +36606,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
@@ -36281,7 +36625,7 @@
       <c r="D1" s="10"/>
       <c r="E1" s="10"/>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="28" t="s">
         <v>826</v>
       </c>
@@ -36298,7 +36642,7 @@
         <v>830</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="91.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="30" t="s">
         <v>831</v>
       </c>
@@ -36315,7 +36659,7 @@
         <v>835</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="30" t="s">
         <v>836</v>
       </c>
@@ -36349,7 +36693,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="30" t="s">
         <v>844</v>
       </c>
@@ -36360,98 +36704,98 @@
         <v>846</v>
       </c>
       <c r="D6" s="29" t="s">
-        <v>844</v>
+        <v>847</v>
       </c>
       <c r="E6" s="29" t="s">
-        <v>847</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>848</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="30" t="s">
-        <v>848</v>
+        <v>849</v>
       </c>
       <c r="B7" s="29" t="s">
         <v>832</v>
       </c>
       <c r="C7" s="29" t="s">
-        <v>849</v>
+        <v>850</v>
       </c>
       <c r="D7" s="29" t="s">
-        <v>850</v>
+        <v>851</v>
       </c>
       <c r="E7" s="29" t="s">
-        <v>851</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>852</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="30" t="s">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="B8" s="29" t="s">
-        <v>853</v>
+        <v>854</v>
       </c>
       <c r="C8" s="29" t="s">
-        <v>854</v>
+        <v>855</v>
       </c>
       <c r="D8" s="29" t="s">
-        <v>855</v>
+        <v>856</v>
       </c>
       <c r="E8" s="29" t="s">
-        <v>856</v>
+        <v>857</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="30" t="s">
-        <v>857</v>
+        <v>858</v>
       </c>
       <c r="B9" s="29" t="s">
         <v>832</v>
       </c>
       <c r="C9" s="29" t="s">
-        <v>858</v>
+        <v>859</v>
       </c>
       <c r="D9" s="29" t="s">
-        <v>859</v>
+        <v>860</v>
       </c>
       <c r="E9" s="29" t="s">
-        <v>860</v>
+        <v>861</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="30" t="s">
-        <v>861</v>
+        <v>862</v>
       </c>
       <c r="B10" s="29" t="s">
         <v>832</v>
       </c>
       <c r="C10" s="29" t="s">
-        <v>862</v>
+        <v>863</v>
       </c>
       <c r="D10" s="29" t="s">
-        <v>863</v>
+        <v>864</v>
       </c>
       <c r="E10" s="29" t="s">
-        <v>860</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>861</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="30" t="s">
-        <v>864</v>
+        <v>865</v>
       </c>
       <c r="B11" s="29" t="s">
         <v>832</v>
       </c>
       <c r="C11" s="29" t="s">
-        <v>865</v>
+        <v>866</v>
       </c>
       <c r="D11" s="29" t="s">
-        <v>866</v>
+        <v>867</v>
       </c>
       <c r="E11" s="29" t="s">
-        <v>867</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="30" t="s">
         <v>24</v>
       </c>
@@ -36459,159 +36803,159 @@
         <v>832</v>
       </c>
       <c r="C12" s="29" t="s">
-        <v>868</v>
+        <v>869</v>
       </c>
       <c r="D12" s="29" t="s">
-        <v>869</v>
+        <v>870</v>
       </c>
       <c r="E12" s="29" t="s">
-        <v>870</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>871</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="78.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="30" t="s">
-        <v>871</v>
+        <v>872</v>
       </c>
       <c r="B13" s="29" t="s">
-        <v>872</v>
+        <v>873</v>
       </c>
       <c r="C13" s="29" t="s">
+        <v>874</v>
+      </c>
+      <c r="D13" s="29" t="s">
+        <v>875</v>
+      </c>
+      <c r="E13" s="29" t="s">
+        <v>876</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="30" t="s">
+        <v>877</v>
+      </c>
+      <c r="B14" s="29" t="s">
         <v>873</v>
       </c>
-      <c r="D13" s="29" t="s">
-        <v>874</v>
-      </c>
-      <c r="E13" s="29" t="s">
-        <v>875</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="30" t="s">
-        <v>876</v>
-      </c>
-      <c r="B14" s="29" t="s">
-        <v>872</v>
-      </c>
       <c r="C14" s="29" t="s">
-        <v>877</v>
+        <v>878</v>
       </c>
       <c r="D14" s="29" t="s">
-        <v>878</v>
+        <v>879</v>
       </c>
       <c r="E14" s="29" t="s">
-        <v>879</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>880</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="30" t="s">
-        <v>880</v>
+        <v>881</v>
       </c>
       <c r="B15" s="29" t="s">
-        <v>872</v>
+        <v>873</v>
       </c>
       <c r="C15" s="29" t="s">
-        <v>881</v>
+        <v>882</v>
       </c>
       <c r="D15" s="29" t="s">
-        <v>882</v>
+        <v>883</v>
       </c>
       <c r="E15" s="29" t="s">
-        <v>883</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>884</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="30" t="s">
-        <v>884</v>
+        <v>885</v>
       </c>
       <c r="B16" s="29" t="s">
-        <v>885</v>
+        <v>886</v>
       </c>
       <c r="C16" s="29" t="s">
-        <v>886</v>
+        <v>887</v>
       </c>
       <c r="D16" s="29" t="s">
-        <v>887</v>
+        <v>888</v>
       </c>
       <c r="E16" s="29" t="s">
-        <v>888</v>
+        <v>889</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="30" t="s">
-        <v>889</v>
+        <v>890</v>
       </c>
       <c r="B17" s="29" t="s">
         <v>832</v>
       </c>
       <c r="C17" s="29" t="s">
-        <v>890</v>
+        <v>891</v>
       </c>
       <c r="D17" s="29" t="s">
         <v>126</v>
       </c>
       <c r="E17" s="29" t="s">
-        <v>891</v>
+        <v>892</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="30" t="s">
-        <v>892</v>
+        <v>893</v>
       </c>
       <c r="B18" s="29" t="s">
         <v>832</v>
       </c>
       <c r="C18" s="29" t="s">
-        <v>893</v>
+        <v>894</v>
       </c>
       <c r="D18" s="29" t="s">
         <v>126</v>
       </c>
       <c r="E18" s="29" t="s">
-        <v>894</v>
+        <v>895</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="30" t="s">
-        <v>895</v>
+        <v>896</v>
       </c>
       <c r="B19" s="29" t="s">
         <v>832</v>
       </c>
       <c r="C19" s="29" t="s">
-        <v>896</v>
+        <v>897</v>
       </c>
       <c r="D19" s="29" t="s">
         <v>126</v>
       </c>
       <c r="E19" s="29" t="s">
-        <v>897</v>
+        <v>898</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="30" t="s">
-        <v>898</v>
+        <v>899</v>
       </c>
       <c r="B20" s="29" t="s">
         <v>832</v>
       </c>
       <c r="C20" s="29" t="s">
-        <v>899</v>
+        <v>900</v>
       </c>
       <c r="D20" s="29" t="s">
         <v>126</v>
       </c>
       <c r="E20" s="29" t="s">
-        <v>894</v>
+        <v>895</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>900</v>
+        <v>901</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="61" t="s">
-        <v>901</v>
+        <v>902</v>
       </c>
       <c r="B23" s="61"/>
       <c r="C23" s="61"/>
@@ -36620,7 +36964,7 @@
     </row>
     <row r="24" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="61" t="s">
-        <v>902</v>
+        <v>903</v>
       </c>
       <c r="B24" s="61"/>
       <c r="C24" s="61"/>
@@ -36629,7 +36973,7 @@
     </row>
     <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="61" t="s">
-        <v>903</v>
+        <v>904</v>
       </c>
       <c r="B25" s="61"/>
       <c r="C25" s="61"/>
@@ -36638,7 +36982,7 @@
     </row>
     <row r="26" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="61" t="s">
-        <v>904</v>
+        <v>905</v>
       </c>
       <c r="B26" s="61"/>
       <c r="C26" s="61"/>
@@ -36647,20 +36991,30 @@
     </row>
     <row r="27" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="61" t="s">
-        <v>905</v>
+        <v>906</v>
       </c>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
       <c r="D27" s="61"/>
       <c r="E27" s="61"/>
     </row>
+    <row r="28" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="61" t="s">
+        <v>907</v>
+      </c>
+      <c r="B28" s="61"/>
+      <c r="C28" s="61"/>
+      <c r="D28" s="61"/>
+      <c r="E28" s="61"/>
+    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="A23:E23"/>
     <mergeCell ref="A24:E24"/>
     <mergeCell ref="A25:E25"/>
     <mergeCell ref="A26:E26"/>
     <mergeCell ref="A27:E27"/>
+    <mergeCell ref="A28:E28"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -36677,7 +37031,448 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:C42"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="60"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="9" t="s">
+        <v>908</v>
+      </c>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+    </row>
+    <row r="2" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>909</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="28" t="s">
+        <v>910</v>
+      </c>
+      <c r="B4" s="28" t="s">
+        <v>911</v>
+      </c>
+      <c r="C4" s="28" t="s">
+        <v>912</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="30" t="s">
+        <v>172</v>
+      </c>
+      <c r="B5" s="31" t="s">
+        <v>913</v>
+      </c>
+      <c r="C5" s="29" t="s">
+        <v>914</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="30" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="31" t="s">
+        <v>915</v>
+      </c>
+      <c r="C6" s="29" t="s">
+        <v>916</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="30" t="s">
+        <v>917</v>
+      </c>
+      <c r="B7" s="31" t="s">
+        <v>918</v>
+      </c>
+      <c r="C7" s="29" t="s">
+        <v>919</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="30" t="s">
+        <v>137</v>
+      </c>
+      <c r="B8" s="31" t="s">
+        <v>920</v>
+      </c>
+      <c r="C8" s="29" t="s">
+        <v>921</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="30" t="s">
+        <v>922</v>
+      </c>
+      <c r="B9" s="31" t="s">
+        <v>923</v>
+      </c>
+      <c r="C9" s="29" t="s">
+        <v>924</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="30" t="s">
+        <v>925</v>
+      </c>
+      <c r="B10" s="31" t="s">
+        <v>926</v>
+      </c>
+      <c r="C10" s="29" t="s">
+        <v>927</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="28" t="s">
+        <v>35</v>
+      </c>
+      <c r="B12" s="28" t="s">
+        <v>928</v>
+      </c>
+      <c r="C12" s="28" t="s">
+        <v>929</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="30" t="s">
+        <v>124</v>
+      </c>
+      <c r="B13" s="31" t="s">
+        <v>930</v>
+      </c>
+      <c r="C13" s="29" t="s">
+        <v>931</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="30" t="s">
+        <v>131</v>
+      </c>
+      <c r="B14" s="31" t="s">
+        <v>932</v>
+      </c>
+      <c r="C14" s="29" t="s">
+        <v>933</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="30" t="s">
+        <v>135</v>
+      </c>
+      <c r="B15" s="31" t="s">
+        <v>934</v>
+      </c>
+      <c r="C15" s="29" t="s">
+        <v>935</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="30" t="s">
+        <v>140</v>
+      </c>
+      <c r="B16" s="31" t="s">
+        <v>936</v>
+      </c>
+      <c r="C16" s="29" t="s">
+        <v>937</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="30" t="s">
+        <v>145</v>
+      </c>
+      <c r="B17" s="31" t="s">
+        <v>938</v>
+      </c>
+      <c r="C17" s="29" t="s">
+        <v>939</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="30" t="s">
+        <v>150</v>
+      </c>
+      <c r="B18" s="31" t="s">
+        <v>940</v>
+      </c>
+      <c r="C18" s="29" t="s">
+        <v>941</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="30" t="s">
+        <v>156</v>
+      </c>
+      <c r="B19" s="31" t="s">
+        <v>942</v>
+      </c>
+      <c r="C19" s="29" t="s">
+        <v>943</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="129" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="B20" s="31" t="s">
+        <v>944</v>
+      </c>
+      <c r="C20" s="29" t="s">
+        <v>945</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="30" t="s">
+        <v>168</v>
+      </c>
+      <c r="B21" s="31" t="s">
+        <v>946</v>
+      </c>
+      <c r="C21" s="29" t="s">
+        <v>947</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="78.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="30" t="s">
+        <v>173</v>
+      </c>
+      <c r="B22" s="31" t="s">
+        <v>948</v>
+      </c>
+      <c r="C22" s="29" t="s">
+        <v>949</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="78.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="30" t="s">
+        <v>180</v>
+      </c>
+      <c r="B23" s="31" t="s">
+        <v>950</v>
+      </c>
+      <c r="C23" s="29" t="s">
+        <v>951</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="78.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="30" t="s">
+        <v>185</v>
+      </c>
+      <c r="B24" s="31" t="s">
+        <v>952</v>
+      </c>
+      <c r="C24" s="29" t="s">
+        <v>953</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="141" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="30" t="s">
+        <v>189</v>
+      </c>
+      <c r="B25" s="31" t="s">
+        <v>954</v>
+      </c>
+      <c r="C25" s="29" t="s">
+        <v>955</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="30" t="s">
+        <v>195</v>
+      </c>
+      <c r="B26" s="31" t="s">
+        <v>956</v>
+      </c>
+      <c r="C26" s="29"/>
+    </row>
+    <row r="27" customFormat="false" ht="141" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="30" t="s">
+        <v>200</v>
+      </c>
+      <c r="B27" s="31" t="s">
+        <v>957</v>
+      </c>
+      <c r="C27" s="29" t="s">
+        <v>958</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="78.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="30" t="s">
+        <v>205</v>
+      </c>
+      <c r="B28" s="31" t="s">
+        <v>952</v>
+      </c>
+      <c r="C28" s="29" t="s">
+        <v>959</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="78.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="30" t="s">
+        <v>207</v>
+      </c>
+      <c r="B29" s="31" t="s">
+        <v>952</v>
+      </c>
+      <c r="C29" s="29"/>
+    </row>
+    <row r="30" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="30" t="s">
+        <v>210</v>
+      </c>
+      <c r="B30" s="31" t="s">
+        <v>960</v>
+      </c>
+      <c r="C30" s="29"/>
+    </row>
+    <row r="31" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="30" t="s">
+        <v>213</v>
+      </c>
+      <c r="B31" s="31" t="s">
+        <v>961</v>
+      </c>
+      <c r="C31" s="29"/>
+    </row>
+    <row r="32" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="30" t="s">
+        <v>219</v>
+      </c>
+      <c r="B32" s="31" t="s">
+        <v>962</v>
+      </c>
+      <c r="C32" s="29" t="s">
+        <v>963</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="30" t="s">
+        <v>224</v>
+      </c>
+      <c r="B33" s="31" t="s">
+        <v>964</v>
+      </c>
+      <c r="C33" s="29" t="s">
+        <v>965</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="30" t="s">
+        <v>226</v>
+      </c>
+      <c r="B34" s="31" t="s">
+        <v>966</v>
+      </c>
+      <c r="C34" s="29" t="s">
+        <v>967</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="30" t="s">
+        <v>229</v>
+      </c>
+      <c r="B35" s="31" t="s">
+        <v>968</v>
+      </c>
+      <c r="C35" s="29"/>
+    </row>
+    <row r="36" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="30" t="s">
+        <v>234</v>
+      </c>
+      <c r="B36" s="31" t="s">
+        <v>969</v>
+      </c>
+      <c r="C36" s="29"/>
+    </row>
+    <row r="37" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="30" t="s">
+        <v>237</v>
+      </c>
+      <c r="B37" s="31" t="s">
+        <v>970</v>
+      </c>
+      <c r="C37" s="29"/>
+    </row>
+    <row r="38" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="30" t="s">
+        <v>242</v>
+      </c>
+      <c r="B38" s="31" t="s">
+        <v>971</v>
+      </c>
+      <c r="C38" s="29"/>
+    </row>
+    <row r="39" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="30" t="s">
+        <v>244</v>
+      </c>
+      <c r="B39" s="31" t="s">
+        <v>972</v>
+      </c>
+      <c r="C39" s="29" t="s">
+        <v>973</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="78.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="30" t="s">
+        <v>249</v>
+      </c>
+      <c r="B40" s="31" t="s">
+        <v>974</v>
+      </c>
+      <c r="C40" s="29"/>
+    </row>
+    <row r="41" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="30" t="s">
+        <v>255</v>
+      </c>
+      <c r="B41" s="31" t="s">
+        <v>975</v>
+      </c>
+      <c r="C41" s="29" t="s">
+        <v>976</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="78.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="30" t="s">
+        <v>260</v>
+      </c>
+      <c r="B42" s="31" t="s">
+        <v>977</v>
+      </c>
+      <c r="C42" s="29" t="s">
+        <v>978</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
@@ -36688,7 +37483,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>906</v>
+        <v>979</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -36696,470 +37491,481 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="62" t="s">
-        <v>907</v>
+        <v>980</v>
       </c>
       <c r="B2" s="62" t="s">
-        <v>908</v>
+        <v>981</v>
       </c>
       <c r="C2" s="62" t="s">
-        <v>909</v>
+        <v>982</v>
       </c>
       <c r="D2" s="62" t="s">
-        <v>910</v>
+        <v>983</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="30" t="s">
-        <v>911</v>
+        <v>984</v>
       </c>
       <c r="B3" s="29" t="s">
-        <v>912</v>
+        <v>985</v>
       </c>
       <c r="C3" s="29" t="s">
-        <v>913</v>
+        <v>986</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="78.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="30" t="s">
-        <v>911</v>
+        <v>984</v>
       </c>
       <c r="B4" s="29" t="s">
-        <v>914</v>
+        <v>987</v>
       </c>
       <c r="C4" s="29" t="s">
-        <v>915</v>
+        <v>988</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="30" t="s">
-        <v>916</v>
+        <v>989</v>
       </c>
       <c r="B5" s="29" t="s">
-        <v>917</v>
+        <v>990</v>
       </c>
       <c r="C5" s="29" t="s">
-        <v>918</v>
+        <v>991</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="30" t="s">
-        <v>919</v>
+        <v>992</v>
       </c>
       <c r="B6" s="29" t="s">
-        <v>920</v>
+        <v>993</v>
       </c>
       <c r="C6" s="29" t="s">
-        <v>921</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>994</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="30" t="s">
-        <v>922</v>
+        <v>995</v>
       </c>
       <c r="B7" s="29" t="s">
-        <v>923</v>
+        <v>996</v>
       </c>
       <c r="C7" s="29" t="s">
-        <v>924</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
-        <v>925</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="30" t="s">
-        <v>124</v>
-      </c>
-      <c r="B10" s="29" t="s">
-        <v>128</v>
-      </c>
-      <c r="C10" s="29" t="s">
-        <v>129</v>
-      </c>
-      <c r="D10" s="63" t="s">
-        <v>926</v>
+        <v>997</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="30" t="s">
+        <v>998</v>
+      </c>
+      <c r="B8" s="29" t="s">
+        <v>999</v>
+      </c>
+      <c r="C8" s="29" t="s">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="s">
+        <v>1001</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="30" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="B11" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="C11" s="29"/>
+        <v>128</v>
+      </c>
+      <c r="C11" s="29" t="s">
+        <v>129</v>
+      </c>
       <c r="D11" s="63" t="s">
-        <v>927</v>
+        <v>1002</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="30" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="B12" s="29" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="C12" s="29"/>
       <c r="D12" s="63" t="s">
-        <v>928</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>1003</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="30" t="s">
+        <v>135</v>
+      </c>
+      <c r="B13" s="29" t="s">
+        <v>139</v>
+      </c>
+      <c r="C13" s="29"/>
+      <c r="D13" s="63" t="s">
+        <v>1004</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="30" t="s">
         <v>140</v>
       </c>
-      <c r="B13" s="29" t="s">
+      <c r="B14" s="29" t="s">
         <v>143</v>
       </c>
-      <c r="C13" s="29" t="s">
+      <c r="C14" s="29" t="s">
         <v>144</v>
       </c>
-      <c r="D13" s="63" t="s">
-        <v>929</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="30" t="s">
+      <c r="D14" s="63" t="s">
+        <v>1005</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="30" t="s">
         <v>145</v>
       </c>
-      <c r="B14" s="29" t="s">
+      <c r="B15" s="29" t="s">
         <v>149</v>
       </c>
-      <c r="C14" s="29"/>
-      <c r="D14" s="63" t="s">
-        <v>930</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="30" t="s">
+      <c r="C15" s="29"/>
+      <c r="D15" s="63" t="s">
+        <v>1006</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="30" t="s">
         <v>150</v>
       </c>
-      <c r="B15" s="29" t="s">
+      <c r="B16" s="29" t="s">
         <v>154</v>
       </c>
-      <c r="C15" s="29" t="s">
+      <c r="C16" s="29" t="s">
         <v>155</v>
       </c>
-      <c r="D15" s="63" t="s">
-        <v>931</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="30" t="s">
+      <c r="D16" s="63" t="s">
+        <v>1007</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="30" t="s">
         <v>156</v>
       </c>
-      <c r="B16" s="29" t="s">
+      <c r="B17" s="29" t="s">
         <v>159</v>
       </c>
-      <c r="C16" s="29" t="s">
+      <c r="C17" s="29" t="s">
         <v>160</v>
       </c>
-      <c r="D16" s="63" t="s">
-        <v>932</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="91.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="30" t="s">
+      <c r="D17" s="63" t="s">
+        <v>1008</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="91.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="30" t="s">
         <v>161</v>
       </c>
-      <c r="B17" s="29" t="s">
+      <c r="B18" s="29" t="s">
         <v>166</v>
       </c>
-      <c r="C17" s="29" t="s">
+      <c r="C18" s="29" t="s">
         <v>167</v>
       </c>
-      <c r="D17" s="63" t="s">
-        <v>933</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="30" t="s">
+      <c r="D18" s="63" t="s">
+        <v>1009</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="30" t="s">
         <v>168</v>
       </c>
-      <c r="B18" s="29" t="s">
+      <c r="B19" s="29" t="s">
         <v>170</v>
       </c>
-      <c r="C18" s="29" t="s">
+      <c r="C19" s="29" t="s">
         <v>171</v>
       </c>
-      <c r="D18" s="63" t="s">
-        <v>934</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="129" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="30" t="s">
+      <c r="D19" s="63" t="s">
+        <v>1010</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="129" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="30" t="s">
         <v>173</v>
       </c>
-      <c r="B19" s="29" t="s">
+      <c r="B20" s="29" t="s">
         <v>178</v>
       </c>
-      <c r="C19" s="29" t="s">
+      <c r="C20" s="29" t="s">
         <v>179</v>
       </c>
-      <c r="D19" s="63" t="s">
-        <v>935</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="91.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="30" t="s">
+      <c r="D20" s="63" t="s">
+        <v>1011</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="91.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="30" t="s">
         <v>180</v>
       </c>
-      <c r="B20" s="29" t="s">
+      <c r="B21" s="29" t="s">
         <v>184</v>
-      </c>
-      <c r="C20" s="29"/>
-      <c r="D20" s="63" t="s">
-        <v>936</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="129" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="30" t="s">
-        <v>185</v>
-      </c>
-      <c r="B21" s="29" t="s">
-        <v>188</v>
       </c>
       <c r="C21" s="29"/>
       <c r="D21" s="63" t="s">
-        <v>937</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="116.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="129" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="30" t="s">
+        <v>185</v>
+      </c>
+      <c r="B22" s="29" t="s">
+        <v>188</v>
+      </c>
+      <c r="C22" s="29"/>
+      <c r="D22" s="63" t="s">
+        <v>1013</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="116.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="30" t="s">
         <v>189</v>
       </c>
-      <c r="B22" s="29" t="s">
+      <c r="B23" s="29" t="s">
         <v>193</v>
       </c>
-      <c r="C22" s="29" t="s">
+      <c r="C23" s="29" t="s">
         <v>194</v>
       </c>
-      <c r="D22" s="63" t="s">
-        <v>938</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="178.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="30" t="s">
+      <c r="D23" s="63" t="s">
+        <v>1014</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="178.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="30" t="s">
         <v>195</v>
       </c>
-      <c r="B23" s="29" t="s">
+      <c r="B24" s="29" t="s">
         <v>198</v>
       </c>
-      <c r="C23" s="29" t="s">
+      <c r="C24" s="29" t="s">
         <v>199</v>
       </c>
-      <c r="D23" s="63" t="s">
-        <v>939</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="141" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="30" t="s">
+      <c r="D24" s="63" t="s">
+        <v>1015</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="141" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="30" t="s">
         <v>200</v>
       </c>
-      <c r="B24" s="29" t="s">
+      <c r="B25" s="29" t="s">
         <v>203</v>
       </c>
-      <c r="C24" s="29" t="s">
+      <c r="C25" s="29" t="s">
         <v>204</v>
       </c>
-      <c r="D24" s="63" t="s">
-        <v>940</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="30" t="s">
-        <v>205</v>
-      </c>
-      <c r="B25" s="29" t="s">
-        <v>206</v>
-      </c>
-      <c r="C25" s="29"/>
       <c r="D25" s="63" t="s">
-        <v>941</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="30" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B26" s="29" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C26" s="29"/>
       <c r="D26" s="63" t="s">
-        <v>941</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="30" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="B27" s="29" t="s">
-        <v>942</v>
+        <v>208</v>
       </c>
       <c r="C27" s="29"/>
       <c r="D27" s="63" t="s">
-        <v>943</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="30" t="s">
+        <v>210</v>
+      </c>
+      <c r="B28" s="29" t="s">
+        <v>1018</v>
+      </c>
+      <c r="C28" s="29"/>
+      <c r="D28" s="63" t="s">
+        <v>1019</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="30" t="s">
         <v>213</v>
       </c>
-      <c r="B28" s="29" t="s">
+      <c r="B29" s="29" t="s">
         <v>217</v>
       </c>
-      <c r="C28" s="29" t="s">
+      <c r="C29" s="29" t="s">
         <v>218</v>
       </c>
-      <c r="D28" s="63" t="s">
-        <v>944</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="78.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="30" t="s">
+      <c r="D29" s="63" t="s">
+        <v>1020</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="78.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="30" t="s">
         <v>219</v>
       </c>
-      <c r="B29" s="29" t="s">
+      <c r="B30" s="29" t="s">
         <v>222</v>
       </c>
-      <c r="C29" s="29" t="s">
+      <c r="C30" s="29" t="s">
         <v>223</v>
       </c>
-      <c r="D29" s="63" t="s">
-        <v>945</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="91.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="30" t="s">
+      <c r="D30" s="63" t="s">
+        <v>1021</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="91.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="30" t="s">
         <v>224</v>
       </c>
-      <c r="B30" s="29" t="s">
-        <v>942</v>
-      </c>
-      <c r="C30" s="29"/>
-      <c r="D30" s="63" t="s">
-        <v>946</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="30" t="s">
-        <v>226</v>
-      </c>
       <c r="B31" s="29" t="s">
-        <v>942</v>
+        <v>1018</v>
       </c>
       <c r="C31" s="29"/>
       <c r="D31" s="63" t="s">
-        <v>947</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>1022</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="30" t="s">
+        <v>226</v>
+      </c>
+      <c r="B32" s="29" t="s">
+        <v>1018</v>
+      </c>
+      <c r="C32" s="29"/>
+      <c r="D32" s="63" t="s">
+        <v>1023</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="30" t="s">
         <v>229</v>
       </c>
-      <c r="B32" s="29" t="s">
+      <c r="B33" s="29" t="s">
         <v>232</v>
       </c>
-      <c r="C32" s="29" t="s">
+      <c r="C33" s="29" t="s">
         <v>233</v>
       </c>
-      <c r="D32" s="63" t="s">
-        <v>948</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="30" t="s">
+      <c r="D33" s="63" t="s">
+        <v>1024</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="30" t="s">
         <v>234</v>
       </c>
-      <c r="B33" s="29" t="s">
+      <c r="B34" s="29" t="s">
         <v>236</v>
       </c>
-      <c r="C33" s="29"/>
-      <c r="D33" s="63" t="s">
-        <v>949</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="30" t="s">
+      <c r="C34" s="29"/>
+      <c r="D34" s="63" t="s">
+        <v>1025</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="30" t="s">
         <v>237</v>
       </c>
-      <c r="B34" s="29" t="s">
-        <v>942</v>
-      </c>
-      <c r="C34" s="29" t="s">
+      <c r="B35" s="29" t="s">
+        <v>1018</v>
+      </c>
+      <c r="C35" s="29" t="s">
         <v>241</v>
       </c>
-      <c r="D34" s="63" t="s">
-        <v>950</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="30" t="s">
+      <c r="D35" s="63" t="s">
+        <v>1026</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="30" t="s">
         <v>242</v>
       </c>
-      <c r="B35" s="29" t="s">
-        <v>942</v>
-      </c>
-      <c r="C35" s="29"/>
-      <c r="D35" s="63" t="s">
-        <v>951</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="30" t="s">
+      <c r="B36" s="29" t="s">
+        <v>1018</v>
+      </c>
+      <c r="C36" s="29"/>
+      <c r="D36" s="63" t="s">
+        <v>1027</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="30" t="s">
         <v>244</v>
       </c>
-      <c r="B36" s="29" t="s">
+      <c r="B37" s="29" t="s">
         <v>247</v>
       </c>
-      <c r="C36" s="29" t="s">
+      <c r="C37" s="29" t="s">
         <v>248</v>
       </c>
-      <c r="D36" s="63" t="s">
-        <v>952</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="30" t="s">
+      <c r="D37" s="63" t="s">
+        <v>1028</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="30" t="s">
         <v>249</v>
       </c>
-      <c r="B37" s="29" t="s">
+      <c r="B38" s="29" t="s">
         <v>252</v>
       </c>
-      <c r="C37" s="29" t="s">
+      <c r="C38" s="29" t="s">
         <v>253</v>
       </c>
-      <c r="D37" s="63" t="s">
-        <v>953</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="30" t="s">
+      <c r="D38" s="63" t="s">
+        <v>1029</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="30" t="s">
         <v>255</v>
       </c>
-      <c r="B38" s="29" t="s">
+      <c r="B39" s="29" t="s">
         <v>258</v>
       </c>
-      <c r="C38" s="29" t="s">
+      <c r="C39" s="29" t="s">
         <v>259</v>
       </c>
-      <c r="D38" s="63" t="s">
-        <v>954</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="129" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="30" t="s">
+      <c r="D39" s="63" t="s">
+        <v>1030</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="129" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="30" t="s">
         <v>260</v>
       </c>
-      <c r="B39" s="29" t="s">
+      <c r="B40" s="29" t="s">
         <v>264</v>
       </c>
-      <c r="C39" s="29"/>
-      <c r="D39" s="63" t="s">
-        <v>955</v>
+      <c r="C40" s="29"/>
+      <c r="D40" s="63" t="s">
+        <v>1031</v>
       </c>
     </row>
   </sheetData>

</xml_diff>